<commit_message>
New Service Manager SPA
</commit_message>
<xml_diff>
--- a/tables/xls/it/70_Volontari preaccreditati.xlsx
+++ b/tables/xls/it/70_Volontari preaccreditati.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="51">
   <si>
     <t>CODICE FISCALE</t>
   </si>
@@ -145,9 +145,6 @@
   </si>
   <si>
     <t>PROV.</t>
-  </si>
-  <si>
-    <t>Nuovo campo</t>
   </si>
   <si>
     <t>Testo - Elenco di valori</t>
@@ -709,7 +706,7 @@
         <v>7</v>
       </c>
       <c r="J3" t="s">
-        <v>43</v>
+        <v>8</v>
       </c>
       <c r="K3" t="s">
         <v>9</v>
@@ -718,7 +715,7 @@
         <v>10</v>
       </c>
       <c r="M3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="N3" t="s">
         <v>12</v>
@@ -759,16 +756,16 @@
         <v>38</v>
       </c>
       <c r="K4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="M4" t="s">
         <v>38</v>
       </c>
       <c r="N4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="O4" t="s">
         <v>38</v>
@@ -779,13 +776,13 @@
         <v>17</v>
       </c>
       <c r="K5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="L5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="N5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -1061,7 +1058,7 @@
         <v>29</v>
       </c>
       <c r="C17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:15">
@@ -1069,7 +1066,7 @@
         <v>30</v>
       </c>
       <c r="B18" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="19" spans="1:15">
@@ -1077,7 +1074,7 @@
         <v>31</v>
       </c>
       <c r="B19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="20" spans="1:15">
@@ -1093,7 +1090,7 @@
         <v>33</v>
       </c>
       <c r="B21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:15">
@@ -1125,7 +1122,7 @@
         <v>37</v>
       </c>
       <c r="B25" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>